<commit_message>
Holocene_Volcanoes_volcdef_cfg: updated with more volcanoes
</commit_message>
<xml_diff>
--- a/Holocene_Volcanoes_volcdef_cfg.xlsx
+++ b/Holocene_Volcanoes_volcdef_cfg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/famelung/code/minsar/tools/webconfig/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9186475-2E83-694B-B13D-3BA00B1F36A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6FAB8D8-B8E3-CC4E-99D5-3848DE9A9BD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5060" yWindow="660" windowWidth="29500" windowHeight="19160" xr2:uid="{C0385577-DB88-5B46-BC32-5548AF298521}"/>
+    <workbookView xWindow="3920" yWindow="1900" windowWidth="33620" windowHeight="19280" xr2:uid="{C0385577-DB88-5B46-BC32-5548AF298521}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11924" uniqueCount="2002">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11935" uniqueCount="2013">
   <si>
     <t>Global Volcanism Program - Volcanoes of the World 5.1.0</t>
   </si>
@@ -6042,6 +6042,39 @@
   </si>
   <si>
     <t>Kilauea vertical</t>
+  </si>
+  <si>
+    <t>149.165.154.65/data/HDF5EOS/Lewotolok/miaplpy/overlay.html#/start/-8.2727/123.5110/14.6000?minScale=-1.5&amp;maxScale=1.5&amp;pixelSize=5.5&amp;background=satellite</t>
+  </si>
+  <si>
+    <t>http://149.165.154.65/data/HDF5EOS/Lewotobi/miaplpy/overlay.html#/start/-8.5402/122.7753/13.5@minScale=-1.5&amp;maxScale=1.5</t>
+  </si>
+  <si>
+    <t>http://149.165.154.65/data/HDF5EOS/Kerinci/miaplpy/overlay.html#/start/-1.696/101.270/14.4?minScale=-0.8&amp;maxScale=0.8&amp;background=satellite</t>
+  </si>
+  <si>
+    <t>http://149.165.153.50/start/-8.2450/117.9958/12.5292?flyToDatasetCenter=false&amp;startDataset=S1_asc_083_miaplpy_20141023_20250215_S0836E11794_S0832E11809_S0817E11806_S0820E11792_filtDel4DS&amp;minScale=-3&amp;maxScale=3&amp;startDate=20141023&amp;endDate=20250215&amp;pixelSize=2.1&amp;background=satellite</t>
+  </si>
+  <si>
+    <t>http://149.165.154.65/data/HDF5EOS/Rinjani/miaplpy/overlay.html#/?minScale=-2&amp;maxScale=2</t>
+  </si>
+  <si>
+    <t>http://149.165.154.65/data/HDF5EOS/Agung/miaplpy/overlay.html#/?minScale=-2&amp;maxScale=2</t>
+  </si>
+  <si>
+    <t>http://149.165.154.65/data/HDF5EOS/Bulusan/miaplpy/overlay.html#/?minScale=-2&amp;maxScale=2&amp;background=satellite</t>
+  </si>
+  <si>
+    <t>http://149.165.154.65/data/HDF5EOS/Merapi/miaplpy/overlay.html#/?minScale=-3&amp;maxScale=3&amp;background=satellite</t>
+  </si>
+  <si>
+    <t>http://149.165.154.65/data/HDF5EOS/Mayon/miaplpy/overlay.html#/?minScale=-2&amp;maxScale=2</t>
+  </si>
+  <si>
+    <t>http://149.165.154.65/data/HDF5EOS/Sinabung/miaplpy/overlay.html#/?minScale=-5&amp;maxScale=5&amp;background=satellite</t>
+  </si>
+  <si>
+    <t>http://149.165.154.65/data/HDF5EOS/Semeru/miaplpy/overlay.html#/?minScale=-2&amp;maxScale=2</t>
   </si>
 </sst>
 </file>
@@ -7814,7 +7847,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="b">
         <v>0</v>
       </c>
@@ -7858,7 +7891,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="b">
         <v>0</v>
       </c>
@@ -7902,7 +7935,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="b">
         <v>0</v>
       </c>
@@ -7946,7 +7979,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="b">
         <v>0</v>
       </c>
@@ -7990,7 +8023,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="b">
         <v>0</v>
       </c>
@@ -8034,7 +8067,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="b">
         <v>0</v>
       </c>
@@ -8078,7 +8111,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="b">
         <v>0</v>
       </c>
@@ -8122,7 +8155,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="b">
         <v>0</v>
       </c>
@@ -8166,7 +8199,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="b">
         <v>0</v>
       </c>
@@ -8210,7 +8243,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="b">
         <v>0</v>
       </c>
@@ -8254,7 +8287,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="41" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="b">
         <v>0</v>
       </c>
@@ -8298,7 +8331,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="b">
         <v>0</v>
       </c>
@@ -8342,7 +8375,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="b">
         <v>0</v>
       </c>
@@ -8386,7 +8419,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="44" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="b">
         <v>0</v>
       </c>
@@ -8430,7 +8463,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="b">
         <v>0</v>
       </c>
@@ -8474,7 +8507,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="b">
         <v>0</v>
       </c>
@@ -8518,7 +8551,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="b">
         <v>0</v>
       </c>
@@ -8562,7 +8595,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="b">
         <v>0</v>
       </c>
@@ -8606,7 +8639,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="49" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="b">
         <v>0</v>
       </c>
@@ -8650,7 +8683,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="50" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="b">
         <v>0</v>
       </c>
@@ -8694,7 +8727,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="51" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="b">
         <v>0</v>
       </c>
@@ -8738,7 +8771,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="b">
         <v>0</v>
       </c>
@@ -8782,7 +8815,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="53" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="b">
         <v>0</v>
       </c>
@@ -8826,7 +8859,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="54" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="b">
         <v>0</v>
       </c>
@@ -8870,7 +8903,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="55" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="b">
         <v>0</v>
       </c>
@@ -8914,7 +8947,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="56" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="b">
         <v>0</v>
       </c>
@@ -8958,7 +8991,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="b">
         <v>0</v>
       </c>
@@ -9002,7 +9035,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="b">
         <v>0</v>
       </c>
@@ -9046,7 +9079,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="59" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="b">
         <v>0</v>
       </c>
@@ -9090,7 +9123,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="60" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="b">
         <v>0</v>
       </c>
@@ -9134,7 +9167,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="61" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="b">
         <v>0</v>
       </c>
@@ -9178,7 +9211,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="b">
         <v>0</v>
       </c>
@@ -9222,7 +9255,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="b">
         <v>0</v>
       </c>
@@ -9266,7 +9299,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="64" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="b">
         <v>0</v>
       </c>
@@ -9310,7 +9343,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="65" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="b">
         <v>0</v>
       </c>
@@ -9354,7 +9387,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="66" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="b">
         <v>0</v>
       </c>
@@ -9398,7 +9431,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="67" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="b">
         <v>0</v>
       </c>
@@ -9442,7 +9475,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="68" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="b">
         <v>0</v>
       </c>
@@ -9486,7 +9519,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="69" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="b">
         <v>0</v>
       </c>
@@ -9530,7 +9563,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="70" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="b">
         <v>0</v>
       </c>
@@ -9574,7 +9607,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="71" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="b">
         <v>0</v>
       </c>
@@ -9618,7 +9651,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="72" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="b">
         <v>0</v>
       </c>
@@ -9662,7 +9695,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="73" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="b">
         <v>0</v>
       </c>
@@ -9706,7 +9739,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="74" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="b">
         <v>0</v>
       </c>
@@ -9750,7 +9783,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="75" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="b">
         <v>0</v>
       </c>
@@ -9794,7 +9827,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="76" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="b">
         <v>0</v>
       </c>
@@ -9838,7 +9871,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="77" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="b">
         <v>0</v>
       </c>
@@ -9882,7 +9915,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="78" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="b">
         <v>0</v>
       </c>
@@ -9926,7 +9959,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="79" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="b">
         <v>0</v>
       </c>
@@ -9970,7 +10003,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="80" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="b">
         <v>0</v>
       </c>
@@ -10014,7 +10047,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="81" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="b">
         <v>0</v>
       </c>
@@ -10058,7 +10091,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="82" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="b">
         <v>0</v>
       </c>
@@ -10102,7 +10135,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="83" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="b">
         <v>0</v>
       </c>
@@ -10146,7 +10179,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="84" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="b">
         <v>0</v>
       </c>
@@ -10190,7 +10223,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="85" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="b">
         <v>0</v>
       </c>
@@ -10234,7 +10267,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="86" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="b">
         <v>0</v>
       </c>
@@ -10278,7 +10311,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="87" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="b">
         <v>0</v>
       </c>
@@ -10322,7 +10355,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="88" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="b">
         <v>0</v>
       </c>
@@ -10366,7 +10399,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="89" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="b">
         <v>0</v>
       </c>
@@ -10410,7 +10443,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="90" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="b">
         <v>0</v>
       </c>
@@ -10454,7 +10487,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="91" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="b">
         <v>0</v>
       </c>
@@ -10498,7 +10531,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="92" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="b">
         <v>0</v>
       </c>
@@ -10542,7 +10575,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="93" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="b">
         <v>0</v>
       </c>
@@ -10586,7 +10619,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="94" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="b">
         <v>0</v>
       </c>
@@ -10630,7 +10663,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="95" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="b">
         <v>0</v>
       </c>
@@ -10674,7 +10707,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="96" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="b">
         <v>0</v>
       </c>
@@ -10718,7 +10751,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="97" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="b">
         <v>0</v>
       </c>
@@ -10762,7 +10795,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="98" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="b">
         <v>0</v>
       </c>
@@ -10806,7 +10839,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="99" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="b">
         <v>0</v>
       </c>
@@ -10850,7 +10883,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="100" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="b">
         <v>0</v>
       </c>
@@ -10894,7 +10927,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="101" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="b">
         <v>0</v>
       </c>
@@ -10938,7 +10971,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="102" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="b">
         <v>0</v>
       </c>
@@ -10982,7 +11015,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="103" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="b">
         <v>0</v>
       </c>
@@ -11026,7 +11059,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="104" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="b">
         <v>0</v>
       </c>
@@ -11070,7 +11103,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="105" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="b">
         <v>0</v>
       </c>
@@ -11114,7 +11147,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="106" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="b">
         <v>0</v>
       </c>
@@ -11158,7 +11191,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="107" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="b">
         <v>0</v>
       </c>
@@ -11202,7 +11235,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="108" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="b">
         <v>0</v>
       </c>
@@ -11246,7 +11279,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="109" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="b">
         <v>0</v>
       </c>
@@ -11290,7 +11323,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="110" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="b">
         <v>0</v>
       </c>
@@ -11334,7 +11367,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="111" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="b">
         <v>0</v>
       </c>
@@ -11378,7 +11411,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="112" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="b">
         <v>0</v>
       </c>
@@ -11422,7 +11455,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="113" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="b">
         <v>0</v>
       </c>
@@ -11466,7 +11499,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="114" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="b">
         <v>0</v>
       </c>
@@ -11510,7 +11543,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="115" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="b">
         <v>0</v>
       </c>
@@ -11554,7 +11587,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="116" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="b">
         <v>0</v>
       </c>
@@ -11598,7 +11631,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="117" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="b">
         <v>0</v>
       </c>
@@ -11642,7 +11675,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="118" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="b">
         <v>0</v>
       </c>
@@ -11686,7 +11719,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="119" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="b">
         <v>0</v>
       </c>
@@ -11730,7 +11763,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="120" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="b">
         <v>0</v>
       </c>
@@ -11774,7 +11807,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="121" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="b">
         <v>0</v>
       </c>
@@ -11818,7 +11851,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="122" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="b">
         <v>0</v>
       </c>
@@ -11862,7 +11895,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="123" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="b">
         <v>0</v>
       </c>
@@ -11906,7 +11939,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="124" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="b">
         <v>0</v>
       </c>
@@ -11950,7 +11983,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="125" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="b">
         <v>0</v>
       </c>
@@ -11994,7 +12027,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="126" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="b">
         <v>0</v>
       </c>
@@ -12038,7 +12071,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="127" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="b">
         <v>0</v>
       </c>
@@ -12082,7 +12115,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="128" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="b">
         <v>0</v>
       </c>
@@ -12126,7 +12159,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="129" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="b">
         <v>0</v>
       </c>
@@ -12170,7 +12203,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="130" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="b">
         <v>0</v>
       </c>
@@ -12214,7 +12247,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="131" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="b">
         <v>0</v>
       </c>
@@ -12258,7 +12291,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="132" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="b">
         <v>0</v>
       </c>
@@ -12302,7 +12335,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="133" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="b">
         <v>0</v>
       </c>
@@ -12346,7 +12379,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="134" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="b">
         <v>0</v>
       </c>
@@ -12390,7 +12423,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="135" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="b">
         <v>0</v>
       </c>
@@ -12434,7 +12467,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="136" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="b">
         <v>0</v>
       </c>
@@ -12478,7 +12511,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="137" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="b">
         <v>0</v>
       </c>
@@ -12522,7 +12555,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="138" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="b">
         <v>0</v>
       </c>
@@ -12566,7 +12599,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="139" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="b">
         <v>0</v>
       </c>
@@ -12610,7 +12643,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="140" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="b">
         <v>0</v>
       </c>
@@ -12654,7 +12687,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="141" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="b">
         <v>0</v>
       </c>
@@ -12698,7 +12731,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="142" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="b">
         <v>0</v>
       </c>
@@ -12742,7 +12775,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="143" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="b">
         <v>0</v>
       </c>
@@ -12786,7 +12819,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="144" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="b">
         <v>0</v>
       </c>
@@ -12830,7 +12863,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="145" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="b">
         <v>0</v>
       </c>
@@ -12874,7 +12907,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="146" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="b">
         <v>0</v>
       </c>
@@ -12918,7 +12951,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="147" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="b">
         <v>0</v>
       </c>
@@ -12962,7 +12995,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="148" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="b">
         <v>0</v>
       </c>
@@ -13006,7 +13039,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="149" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="b">
         <v>0</v>
       </c>
@@ -13050,7 +13083,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="150" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="b">
         <v>0</v>
       </c>
@@ -13094,7 +13127,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="151" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="b">
         <v>0</v>
       </c>
@@ -13138,7 +13171,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="152" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="b">
         <v>0</v>
       </c>
@@ -13182,7 +13215,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="153" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="b">
         <v>0</v>
       </c>
@@ -13226,7 +13259,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="154" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="b">
         <v>0</v>
       </c>
@@ -13270,7 +13303,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="155" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="b">
         <v>0</v>
       </c>
@@ -13314,7 +13347,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="156" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="b">
         <v>0</v>
       </c>
@@ -13358,7 +13391,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="157" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="b">
         <v>0</v>
       </c>
@@ -13402,7 +13435,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="158" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="b">
         <v>0</v>
       </c>
@@ -13446,7 +13479,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="159" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="b">
         <v>0</v>
       </c>
@@ -13490,7 +13523,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="160" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="b">
         <v>0</v>
       </c>
@@ -13534,7 +13567,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="161" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="b">
         <v>0</v>
       </c>
@@ -13578,7 +13611,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="162" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="b">
         <v>0</v>
       </c>
@@ -13622,7 +13655,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="163" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163" s="1" t="b">
         <v>0</v>
       </c>
@@ -13666,7 +13699,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="164" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A164" s="1" t="b">
         <v>0</v>
       </c>
@@ -13710,7 +13743,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="165" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A165" s="1" t="b">
         <v>0</v>
       </c>
@@ -13754,7 +13787,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="166" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" s="1" t="b">
         <v>0</v>
       </c>
@@ -13798,7 +13831,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="167" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167" s="1" t="b">
         <v>0</v>
       </c>
@@ -13842,7 +13875,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="168" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A168" s="1" t="b">
         <v>0</v>
       </c>
@@ -13886,7 +13919,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="169" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A169" s="1" t="b">
         <v>0</v>
       </c>
@@ -13930,7 +13963,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="170" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170" s="1" t="b">
         <v>0</v>
       </c>
@@ -13974,7 +14007,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="171" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171" s="1" t="b">
         <v>0</v>
       </c>
@@ -14018,7 +14051,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="172" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="1" t="b">
         <v>0</v>
       </c>
@@ -14062,7 +14095,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="173" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" s="1" t="b">
         <v>0</v>
       </c>
@@ -14106,7 +14139,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="174" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" s="1" t="b">
         <v>0</v>
       </c>
@@ -14150,7 +14183,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="175" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" s="1" t="b">
         <v>0</v>
       </c>
@@ -14194,7 +14227,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="176" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" s="1" t="b">
         <v>0</v>
       </c>
@@ -14238,7 +14271,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="177" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="1" t="b">
         <v>0</v>
       </c>
@@ -14282,7 +14315,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="178" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" s="1" t="b">
         <v>0</v>
       </c>
@@ -14326,7 +14359,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="179" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" s="1" t="b">
         <v>0</v>
       </c>
@@ -14370,7 +14403,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="180" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" s="1" t="b">
         <v>0</v>
       </c>
@@ -14414,7 +14447,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="181" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="1" t="b">
         <v>0</v>
       </c>
@@ -14458,7 +14491,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="182" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" s="1" t="b">
         <v>0</v>
       </c>
@@ -14502,7 +14535,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="183" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" s="1" t="b">
         <v>0</v>
       </c>
@@ -14546,7 +14579,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="184" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184" s="1" t="b">
         <v>0</v>
       </c>
@@ -14590,7 +14623,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="185" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A185" s="1" t="b">
         <v>0</v>
       </c>
@@ -14634,7 +14667,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="186" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186" s="1" t="b">
         <v>0</v>
       </c>
@@ -14678,7 +14711,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="187" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187" s="1" t="b">
         <v>0</v>
       </c>
@@ -14722,7 +14755,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="188" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188" s="1" t="b">
         <v>0</v>
       </c>
@@ -14766,7 +14799,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="189" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A189" s="1" t="b">
         <v>0</v>
       </c>
@@ -14810,7 +14843,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="190" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A190" s="1" t="b">
         <v>0</v>
       </c>
@@ -14854,7 +14887,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="191" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A191" s="1" t="b">
         <v>0</v>
       </c>
@@ -14898,7 +14931,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="192" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A192" s="1" t="b">
         <v>0</v>
       </c>
@@ -14942,7 +14975,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="193" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A193" s="1" t="b">
         <v>0</v>
       </c>
@@ -14986,7 +15019,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="194" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A194" s="1" t="b">
         <v>0</v>
       </c>
@@ -15030,7 +15063,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="195" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A195" s="1" t="b">
         <v>0</v>
       </c>
@@ -15074,7 +15107,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="196" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A196" s="1" t="b">
         <v>0</v>
       </c>
@@ -15118,7 +15151,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="197" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A197" s="1" t="b">
         <v>0</v>
       </c>
@@ -15162,7 +15195,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="198" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A198" s="1" t="b">
         <v>0</v>
       </c>
@@ -15206,7 +15239,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="199" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A199" s="1" t="b">
         <v>0</v>
       </c>
@@ -15250,7 +15283,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="200" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A200" s="1" t="b">
         <v>0</v>
       </c>
@@ -15294,7 +15327,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="201" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A201" s="1" t="b">
         <v>0</v>
       </c>
@@ -15338,7 +15371,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="202" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A202" s="1" t="b">
         <v>0</v>
       </c>
@@ -15382,7 +15415,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="203" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A203" s="1" t="b">
         <v>0</v>
       </c>
@@ -15426,7 +15459,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="204" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A204" s="1" t="b">
         <v>0</v>
       </c>
@@ -15470,7 +15503,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="205" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A205" s="1" t="b">
         <v>0</v>
       </c>
@@ -15514,7 +15547,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="206" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A206" s="1" t="b">
         <v>0</v>
       </c>
@@ -15558,7 +15591,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="207" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A207" s="1" t="b">
         <v>0</v>
       </c>
@@ -15602,7 +15635,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="208" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A208" s="1" t="b">
         <v>0</v>
       </c>
@@ -15646,7 +15679,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="209" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A209" s="1" t="b">
         <v>0</v>
       </c>
@@ -15690,7 +15723,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="210" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A210" s="1" t="b">
         <v>0</v>
       </c>
@@ -15734,7 +15767,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="211" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A211" s="1" t="b">
         <v>0</v>
       </c>
@@ -15778,7 +15811,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="212" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A212" s="1" t="b">
         <v>0</v>
       </c>
@@ -15822,7 +15855,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="213" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A213" s="1" t="b">
         <v>0</v>
       </c>
@@ -15866,7 +15899,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="214" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A214" s="1" t="b">
         <v>0</v>
       </c>
@@ -15910,7 +15943,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="215" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A215" s="1" t="b">
         <v>0</v>
       </c>
@@ -15954,7 +15987,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="216" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A216" s="1" t="b">
         <v>0</v>
       </c>
@@ -15998,7 +16031,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="217" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A217" s="1" t="b">
         <v>0</v>
       </c>
@@ -16042,7 +16075,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="218" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A218" s="1" t="b">
         <v>0</v>
       </c>
@@ -16086,7 +16119,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="219" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A219" s="1" t="b">
         <v>0</v>
       </c>
@@ -16130,7 +16163,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="220" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A220" s="1" t="b">
         <v>0</v>
       </c>
@@ -16174,7 +16207,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="221" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A221" s="1" t="b">
         <v>0</v>
       </c>
@@ -16218,7 +16251,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="222" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A222" s="1" t="b">
         <v>0</v>
       </c>
@@ -16262,7 +16295,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="223" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A223" s="1" t="b">
         <v>0</v>
       </c>
@@ -16306,7 +16339,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="224" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A224" s="1" t="b">
         <v>0</v>
       </c>
@@ -16350,7 +16383,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="225" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A225" s="1" t="b">
         <v>0</v>
       </c>
@@ -16394,7 +16427,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="226" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A226" s="1" t="b">
         <v>0</v>
       </c>
@@ -16438,7 +16471,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="227" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A227" s="1" t="b">
         <v>0</v>
       </c>
@@ -16482,7 +16515,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="228" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A228" s="1" t="b">
         <v>0</v>
       </c>
@@ -16526,7 +16559,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="229" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A229" s="1" t="b">
         <v>0</v>
       </c>
@@ -16570,7 +16603,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="230" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A230" s="1" t="b">
         <v>0</v>
       </c>
@@ -16614,7 +16647,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="231" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A231" s="1" t="b">
         <v>0</v>
       </c>
@@ -16658,7 +16691,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="232" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A232" s="1" t="b">
         <v>0</v>
       </c>
@@ -16702,7 +16735,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="233" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A233" s="1" t="b">
         <v>0</v>
       </c>
@@ -16746,7 +16779,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="234" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A234" s="1" t="b">
         <v>0</v>
       </c>
@@ -16790,7 +16823,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="235" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A235" s="1" t="b">
         <v>0</v>
       </c>
@@ -16834,7 +16867,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="236" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A236" s="1" t="b">
         <v>0</v>
       </c>
@@ -16878,7 +16911,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="237" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A237" s="1" t="b">
         <v>0</v>
       </c>
@@ -16922,7 +16955,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="238" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A238" s="1" t="b">
         <v>0</v>
       </c>
@@ -16966,7 +16999,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="239" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A239" s="1" t="b">
         <v>0</v>
       </c>
@@ -17010,7 +17043,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="240" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A240" s="1" t="b">
         <v>0</v>
       </c>
@@ -17054,7 +17087,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="241" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A241" s="1" t="b">
         <v>0</v>
       </c>
@@ -17098,7 +17131,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="242" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A242" s="1" t="b">
         <v>0</v>
       </c>
@@ -17142,7 +17175,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="243" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A243" s="1" t="b">
         <v>0</v>
       </c>
@@ -17186,7 +17219,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="244" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A244" s="1" t="b">
         <v>0</v>
       </c>
@@ -17230,7 +17263,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="245" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A245" s="1" t="b">
         <v>0</v>
       </c>
@@ -17274,7 +17307,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="246" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A246" s="1" t="b">
         <v>0</v>
       </c>
@@ -17318,7 +17351,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="247" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A247" s="1" t="b">
         <v>0</v>
       </c>
@@ -17362,7 +17395,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="248" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A248" s="1" t="b">
         <v>0</v>
       </c>
@@ -17406,7 +17439,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="249" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A249" s="1" t="b">
         <v>0</v>
       </c>
@@ -17450,7 +17483,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="250" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A250" s="1" t="b">
         <v>0</v>
       </c>
@@ -17494,7 +17527,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="251" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A251" s="1" t="b">
         <v>0</v>
       </c>
@@ -17538,7 +17571,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="252" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A252" s="1" t="b">
         <v>0</v>
       </c>
@@ -17582,7 +17615,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="253" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A253" s="1" t="b">
         <v>0</v>
       </c>
@@ -17626,7 +17659,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="254" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A254" s="1" t="b">
         <v>0</v>
       </c>
@@ -17670,7 +17703,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="255" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A255" s="1" t="b">
         <v>0</v>
       </c>
@@ -17714,7 +17747,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="256" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A256" s="1" t="b">
         <v>0</v>
       </c>
@@ -17758,7 +17791,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="257" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A257" s="1" t="b">
         <v>0</v>
       </c>
@@ -17802,7 +17835,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="258" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A258" s="1" t="b">
         <v>0</v>
       </c>
@@ -17846,7 +17879,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="259" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A259" s="1" t="b">
         <v>0</v>
       </c>
@@ -17890,7 +17923,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="260" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A260" s="1" t="b">
         <v>0</v>
       </c>
@@ -17934,7 +17967,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="261" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A261" s="1" t="b">
         <v>0</v>
       </c>
@@ -17978,7 +18011,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="262" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A262" s="1" t="b">
         <v>0</v>
       </c>
@@ -18022,7 +18055,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="263" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A263" s="1" t="b">
         <v>0</v>
       </c>
@@ -18066,7 +18099,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="264" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A264" s="1" t="b">
         <v>0</v>
       </c>
@@ -18110,7 +18143,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="265" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A265" s="1" t="b">
         <v>0</v>
       </c>
@@ -18154,7 +18187,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="266" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A266" s="1" t="b">
         <v>0</v>
       </c>
@@ -18198,7 +18231,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="267" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A267" s="1" t="b">
         <v>0</v>
       </c>
@@ -18242,7 +18275,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="268" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A268" s="1" t="b">
         <v>0</v>
       </c>
@@ -18286,7 +18319,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="269" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A269" s="1" t="b">
         <v>0</v>
       </c>
@@ -18330,7 +18363,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="270" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A270" s="1" t="b">
         <v>0</v>
       </c>
@@ -18374,7 +18407,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="271" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A271" s="1" t="b">
         <v>0</v>
       </c>
@@ -18418,7 +18451,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="272" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A272" s="1" t="b">
         <v>0</v>
       </c>
@@ -18462,7 +18495,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="273" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A273" s="1" t="b">
         <v>0</v>
       </c>
@@ -18506,7 +18539,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="274" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A274" s="1" t="b">
         <v>0</v>
       </c>
@@ -18550,7 +18583,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="275" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A275" s="1" t="b">
         <v>0</v>
       </c>
@@ -18594,7 +18627,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="276" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A276" s="1" t="b">
         <v>0</v>
       </c>
@@ -18638,7 +18671,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="277" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A277" s="1" t="b">
         <v>0</v>
       </c>
@@ -18682,7 +18715,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="278" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A278" s="1" t="b">
         <v>0</v>
       </c>
@@ -18726,7 +18759,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="279" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A279" s="1" t="b">
         <v>0</v>
       </c>
@@ -18770,7 +18803,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="280" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A280" s="1" t="b">
         <v>0</v>
       </c>
@@ -18814,7 +18847,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="281" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A281" s="1" t="b">
         <v>0</v>
       </c>
@@ -18858,7 +18891,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="282" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A282" s="1" t="b">
         <v>0</v>
       </c>
@@ -18902,7 +18935,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="283" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A283" s="1" t="b">
         <v>0</v>
       </c>
@@ -18946,7 +18979,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="284" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A284" s="1" t="b">
         <v>0</v>
       </c>
@@ -18990,7 +19023,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="285" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A285" s="1" t="b">
         <v>0</v>
       </c>
@@ -19034,7 +19067,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="286" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A286" s="1" t="b">
         <v>0</v>
       </c>
@@ -19078,7 +19111,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="287" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A287" s="1" t="b">
         <v>0</v>
       </c>
@@ -19122,7 +19155,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="288" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A288" s="1" t="b">
         <v>0</v>
       </c>
@@ -19166,7 +19199,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="289" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A289" s="1" t="b">
         <v>0</v>
       </c>
@@ -19210,7 +19243,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="290" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A290" s="1" t="b">
         <v>0</v>
       </c>
@@ -19254,7 +19287,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="291" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A291" s="1" t="b">
         <v>0</v>
       </c>
@@ -19298,7 +19331,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="292" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A292" s="1" t="b">
         <v>0</v>
       </c>
@@ -19342,7 +19375,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="293" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A293" s="1" t="b">
         <v>0</v>
       </c>
@@ -19386,7 +19419,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="294" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A294" s="1" t="b">
         <v>0</v>
       </c>
@@ -19430,7 +19463,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="295" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A295" s="1" t="b">
         <v>0</v>
       </c>
@@ -19474,7 +19507,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="296" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A296" s="1" t="b">
         <v>0</v>
       </c>
@@ -19518,7 +19551,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="297" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A297" s="1" t="b">
         <v>0</v>
       </c>
@@ -19562,7 +19595,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="298" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A298" s="1" t="b">
         <v>0</v>
       </c>
@@ -19606,7 +19639,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="299" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A299" s="1" t="b">
         <v>0</v>
       </c>
@@ -19650,7 +19683,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="300" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A300" s="1" t="b">
         <v>0</v>
       </c>
@@ -19694,7 +19727,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="301" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A301" s="1" t="b">
         <v>0</v>
       </c>
@@ -19738,7 +19771,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="302" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A302" s="1" t="b">
         <v>0</v>
       </c>
@@ -19782,7 +19815,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="303" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A303" s="1" t="b">
         <v>0</v>
       </c>
@@ -19826,7 +19859,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="304" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A304" s="1" t="b">
         <v>0</v>
       </c>
@@ -19870,7 +19903,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="305" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A305" s="1" t="b">
         <v>0</v>
       </c>
@@ -19914,7 +19947,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="306" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A306" s="1" t="b">
         <v>0</v>
       </c>
@@ -19958,7 +19991,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="307" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A307" s="1" t="b">
         <v>0</v>
       </c>
@@ -20002,7 +20035,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="308" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A308" s="1" t="b">
         <v>0</v>
       </c>
@@ -20046,7 +20079,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="309" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A309" s="1" t="b">
         <v>0</v>
       </c>
@@ -20090,7 +20123,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="310" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A310" s="1" t="b">
         <v>0</v>
       </c>
@@ -20134,7 +20167,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="311" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A311" s="1" t="b">
         <v>0</v>
       </c>
@@ -20178,7 +20211,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="312" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A312" s="1" t="b">
         <v>0</v>
       </c>
@@ -20222,7 +20255,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="313" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A313" s="1" t="b">
         <v>0</v>
       </c>
@@ -20266,7 +20299,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="314" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A314" s="1" t="b">
         <v>0</v>
       </c>
@@ -20310,7 +20343,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="315" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="315" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A315" s="1" t="b">
         <v>0</v>
       </c>
@@ -20354,7 +20387,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="316" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="316" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A316" s="1" t="b">
         <v>0</v>
       </c>
@@ -20398,7 +20431,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="317" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A317" s="1" t="b">
         <v>0</v>
       </c>
@@ -20442,7 +20475,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="318" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="318" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A318" s="1" t="b">
         <v>0</v>
       </c>
@@ -20486,7 +20519,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="319" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="319" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A319" s="1" t="b">
         <v>0</v>
       </c>
@@ -20530,7 +20563,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="320" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="320" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A320" s="1" t="b">
         <v>0</v>
       </c>
@@ -20574,7 +20607,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="321" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A321" s="1" t="b">
         <v>0</v>
       </c>
@@ -20618,7 +20651,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="322" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="322" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A322" s="1" t="b">
         <v>0</v>
       </c>
@@ -20662,7 +20695,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="323" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="323" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A323" s="1" t="b">
         <v>0</v>
       </c>
@@ -20706,7 +20739,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="324" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="324" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A324" s="1" t="b">
         <v>0</v>
       </c>
@@ -20750,7 +20783,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="325" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="325" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A325" s="1" t="b">
         <v>0</v>
       </c>
@@ -20794,7 +20827,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="326" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="326" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A326" s="1" t="b">
         <v>0</v>
       </c>
@@ -20838,7 +20871,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="327" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A327" s="1" t="b">
         <v>0</v>
       </c>
@@ -20882,7 +20915,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="328" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="328" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A328" s="1" t="b">
         <v>0</v>
       </c>
@@ -20926,7 +20959,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="329" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="329" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A329" s="1" t="b">
         <v>0</v>
       </c>
@@ -20970,7 +21003,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="330" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="330" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A330" s="1" t="b">
         <v>0</v>
       </c>
@@ -21014,7 +21047,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="331" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="331" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A331" s="1" t="b">
         <v>0</v>
       </c>
@@ -21058,7 +21091,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="332" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="332" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A332" s="1" t="b">
         <v>0</v>
       </c>
@@ -21102,7 +21135,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="333" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="333" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A333" s="1" t="b">
         <v>0</v>
       </c>
@@ -21146,7 +21179,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="334" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="334" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A334" s="1" t="b">
         <v>0</v>
       </c>
@@ -21190,7 +21223,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="335" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="335" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A335" s="1" t="b">
         <v>0</v>
       </c>
@@ -21234,7 +21267,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="336" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A336" s="1" t="b">
         <v>0</v>
       </c>
@@ -21278,7 +21311,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="337" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A337" s="1" t="b">
         <v>0</v>
       </c>
@@ -21322,9 +21355,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="338" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A338" s="1" t="b">
-        <v>0</v>
+    <row r="338" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A338" s="6" t="s">
+        <v>2011</v>
       </c>
       <c r="B338" s="3">
         <v>261080</v>
@@ -21366,7 +21399,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="339" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="339" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A339" s="1" t="b">
         <v>0</v>
       </c>
@@ -21410,7 +21443,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="340" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="340" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A340" s="1" t="b">
         <v>0</v>
       </c>
@@ -21454,7 +21487,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="341" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A341" s="1" t="b">
         <v>0</v>
       </c>
@@ -21498,7 +21531,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="342" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A342" s="1" t="b">
         <v>0</v>
       </c>
@@ -21542,7 +21575,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="343" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A343" s="1" t="b">
         <v>0</v>
       </c>
@@ -21586,7 +21619,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="344" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="344" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A344" s="1" t="b">
         <v>0</v>
       </c>
@@ -21630,7 +21663,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="345" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="345" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A345" s="1" t="b">
         <v>0</v>
       </c>
@@ -21674,7 +21707,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="346" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A346" s="1" t="b">
         <v>0</v>
       </c>
@@ -21718,7 +21751,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="347" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="347" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A347" s="1" t="b">
         <v>0</v>
       </c>
@@ -21762,7 +21795,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="348" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="348" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A348" s="1" t="b">
         <v>0</v>
       </c>
@@ -21806,9 +21839,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="349" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A349" s="1" t="b">
-        <v>0</v>
+    <row r="349" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A349" s="6" t="s">
+        <v>2004</v>
       </c>
       <c r="B349" s="3">
         <v>261170</v>
@@ -21850,7 +21883,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="350" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A350" s="1" t="b">
         <v>0</v>
       </c>
@@ -21894,7 +21927,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="351" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="351" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A351" s="1" t="b">
         <v>0</v>
       </c>
@@ -21938,7 +21971,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="352" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="352" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A352" s="1" t="b">
         <v>0</v>
       </c>
@@ -21982,7 +22015,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="353" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="353" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A353" s="1" t="b">
         <v>0</v>
       </c>
@@ -22026,7 +22059,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="354" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="354" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A354" s="1" t="b">
         <v>0</v>
       </c>
@@ -22070,7 +22103,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="355" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="355" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A355" s="1" t="b">
         <v>0</v>
       </c>
@@ -22114,7 +22147,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="356" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="356" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A356" s="1" t="b">
         <v>0</v>
       </c>
@@ -22158,7 +22191,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="357" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="357" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A357" s="1" t="b">
         <v>0</v>
       </c>
@@ -22202,7 +22235,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="358" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="358" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A358" s="1" t="b">
         <v>0</v>
       </c>
@@ -22246,7 +22279,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="359" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="359" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A359" s="1" t="b">
         <v>0</v>
       </c>
@@ -22290,7 +22323,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="360" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="360" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A360" s="1" t="b">
         <v>0</v>
       </c>
@@ -22334,7 +22367,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="361" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="361" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A361" s="1" t="b">
         <v>0</v>
       </c>
@@ -22378,7 +22411,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="362" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="362" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A362" s="1" t="b">
         <v>0</v>
       </c>
@@ -22422,7 +22455,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="363" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="363" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A363" s="1" t="b">
         <v>0</v>
       </c>
@@ -22466,7 +22499,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="364" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="364" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A364" s="1" t="b">
         <v>0</v>
       </c>
@@ -22510,7 +22543,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="365" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="365" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A365" s="1" t="b">
         <v>0</v>
       </c>
@@ -22554,7 +22587,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="366" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="366" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A366" s="1" t="b">
         <v>0</v>
       </c>
@@ -22598,7 +22631,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="367" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="367" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A367" s="1" t="b">
         <v>0</v>
       </c>
@@ -22642,7 +22675,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="368" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="368" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A368" s="1" t="b">
         <v>0</v>
       </c>
@@ -22686,7 +22719,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="369" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="369" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A369" s="1" t="b">
         <v>0</v>
       </c>
@@ -22730,7 +22763,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="370" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="370" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A370" s="1" t="b">
         <v>0</v>
       </c>
@@ -22774,7 +22807,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="371" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="371" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A371" s="1" t="b">
         <v>0</v>
       </c>
@@ -22818,7 +22851,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="372" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="372" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A372" s="1" t="b">
         <v>0</v>
       </c>
@@ -22862,7 +22895,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="373" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="373" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A373" s="1" t="b">
         <v>0</v>
       </c>
@@ -22906,7 +22939,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="374" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="374" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A374" s="1" t="b">
         <v>0</v>
       </c>
@@ -22950,7 +22983,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="375" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="375" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A375" s="1" t="b">
         <v>0</v>
       </c>
@@ -22994,7 +23027,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="376" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="376" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A376" s="1" t="b">
         <v>0</v>
       </c>
@@ -23038,7 +23071,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="377" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="377" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A377" s="1" t="b">
         <v>0</v>
       </c>
@@ -23126,7 +23159,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="379" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="379" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A379" s="1" t="b">
         <v>0</v>
       </c>
@@ -23170,7 +23203,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="380" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="380" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A380" s="1" t="b">
         <v>0</v>
       </c>
@@ -23214,7 +23247,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="381" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="381" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A381" s="1" t="b">
         <v>0</v>
       </c>
@@ -23303,8 +23336,8 @@
       </c>
     </row>
     <row r="383" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A383" s="1" t="b">
-        <v>0</v>
+      <c r="A383" s="6" t="s">
+        <v>2009</v>
       </c>
       <c r="B383" s="3">
         <v>263250</v>
@@ -23391,8 +23424,8 @@
       </c>
     </row>
     <row r="385" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A385" s="1" t="b">
-        <v>0</v>
+      <c r="A385" s="6" t="s">
+        <v>2012</v>
       </c>
       <c r="B385" s="3">
         <v>263300</v>
@@ -23654,7 +23687,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="391" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="391" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A391" s="1" t="b">
         <v>0</v>
       </c>
@@ -23698,7 +23731,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="392" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="392" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A392" s="1" t="b">
         <v>0</v>
       </c>
@@ -23787,8 +23820,8 @@
       </c>
     </row>
     <row r="394" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A394" s="1" t="b">
-        <v>0</v>
+      <c r="A394" s="6" t="s">
+        <v>2007</v>
       </c>
       <c r="B394" s="3">
         <v>264020</v>
@@ -23831,8 +23864,8 @@
       </c>
     </row>
     <row r="395" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A395" s="1" t="b">
-        <v>0</v>
+      <c r="A395" s="6" t="s">
+        <v>2006</v>
       </c>
       <c r="B395" s="3">
         <v>264030</v>
@@ -23875,8 +23908,8 @@
       </c>
     </row>
     <row r="396" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A396" s="1" t="b">
-        <v>0</v>
+      <c r="A396" s="6" t="s">
+        <v>2005</v>
       </c>
       <c r="B396" s="3">
         <v>264040</v>
@@ -23963,8 +23996,8 @@
       </c>
     </row>
     <row r="398" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A398" s="1" t="b">
-        <v>0</v>
+      <c r="A398" s="6" t="s">
+        <v>2003</v>
       </c>
       <c r="B398" s="3">
         <v>264180</v>
@@ -24006,7 +24039,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="399" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="399" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A399" s="1" t="b">
         <v>0</v>
       </c>
@@ -24050,7 +24083,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="400" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="400" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A400" s="1" t="b">
         <v>0</v>
       </c>
@@ -24094,9 +24127,9 @@
         <v>463</v>
       </c>
     </row>
-    <row r="401" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A401" s="1" t="b">
-        <v>0</v>
+    <row r="401" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A401" s="6" t="s">
+        <v>2002</v>
       </c>
       <c r="B401" s="3">
         <v>264230</v>
@@ -24138,7 +24171,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="402" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="402" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A402" s="1" t="b">
         <v>0</v>
       </c>
@@ -24314,7 +24347,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="406" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="406" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A406" s="1" t="b">
         <v>0</v>
       </c>
@@ -24358,7 +24391,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="407" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="407" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A407" s="1" t="b">
         <v>0</v>
       </c>
@@ -24490,7 +24523,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="410" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="410" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A410" s="1" t="b">
         <v>0</v>
       </c>
@@ -24578,7 +24611,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="412" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="412" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A412" s="1" t="b">
         <v>0</v>
       </c>
@@ -24622,7 +24655,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="413" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="413" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A413" s="1" t="b">
         <v>0</v>
       </c>
@@ -24710,7 +24743,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="415" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="415" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A415" s="1" t="b">
         <v>0</v>
       </c>
@@ -24754,7 +24787,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="416" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="416" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A416" s="1" t="b">
         <v>0</v>
       </c>
@@ -24798,7 +24831,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="417" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="417" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A417" s="1" t="b">
         <v>0</v>
       </c>
@@ -24842,7 +24875,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="418" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="418" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A418" s="1" t="b">
         <v>0</v>
       </c>
@@ -24974,7 +25007,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="421" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="421" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A421" s="1" t="b">
         <v>0</v>
       </c>
@@ -25150,7 +25183,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="425" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="425" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A425" s="1" t="b">
         <v>0</v>
       </c>
@@ -25238,7 +25271,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="427" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="427" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A427" s="1" t="b">
         <v>0</v>
       </c>
@@ -25282,7 +25315,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="428" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="428" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A428" s="1" t="b">
         <v>0</v>
       </c>
@@ -25326,7 +25359,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="429" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="429" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A429" s="1" t="b">
         <v>0</v>
       </c>
@@ -25370,7 +25403,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="430" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="430" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A430" s="1" t="b">
         <v>0</v>
       </c>
@@ -25458,7 +25491,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="432" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="432" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A432" s="1" t="b">
         <v>0</v>
       </c>
@@ -25502,7 +25535,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="433" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="433" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A433" s="1" t="b">
         <v>0</v>
       </c>
@@ -25546,7 +25579,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="434" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="434" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A434" s="1" t="b">
         <v>0</v>
       </c>
@@ -25590,7 +25623,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="435" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="435" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A435" s="1" t="b">
         <v>0</v>
       </c>
@@ -25634,7 +25667,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="436" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="436" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A436" s="1" t="b">
         <v>0</v>
       </c>
@@ -25678,7 +25711,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="437" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="437" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A437" s="1" t="b">
         <v>0</v>
       </c>
@@ -25722,7 +25755,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="438" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="438" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A438" s="1" t="b">
         <v>0</v>
       </c>
@@ -25766,7 +25799,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="439" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="439" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A439" s="1" t="b">
         <v>0</v>
       </c>
@@ -25810,7 +25843,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="440" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="440" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A440" s="1" t="b">
         <v>0</v>
       </c>
@@ -25854,7 +25887,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="441" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="441" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A441" s="1" t="b">
         <v>0</v>
       </c>
@@ -25898,7 +25931,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="442" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="442" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A442" s="1" t="b">
         <v>0</v>
       </c>
@@ -25942,7 +25975,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="443" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="443" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A443" s="1" t="b">
         <v>0</v>
       </c>
@@ -25986,7 +26019,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="444" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="444" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A444" s="1" t="b">
         <v>0</v>
       </c>
@@ -26030,7 +26063,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="445" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="445" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A445" s="1" t="b">
         <v>0</v>
       </c>
@@ -26074,7 +26107,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="446" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="446" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A446" s="1" t="b">
         <v>0</v>
       </c>
@@ -26118,7 +26151,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="447" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="447" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A447" s="1" t="b">
         <v>0</v>
       </c>
@@ -26162,7 +26195,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="448" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="448" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A448" s="1" t="b">
         <v>0</v>
       </c>
@@ -26206,7 +26239,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="449" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="449" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A449" s="1" t="b">
         <v>0</v>
       </c>
@@ -26250,7 +26283,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="450" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="450" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A450" s="1" t="b">
         <v>0</v>
       </c>
@@ -26294,7 +26327,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="451" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="451" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A451" s="1" t="b">
         <v>0</v>
       </c>
@@ -26338,7 +26371,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="452" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="452" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A452" s="1" t="b">
         <v>0</v>
       </c>
@@ -26382,7 +26415,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="453" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="453" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A453" s="1" t="b">
         <v>0</v>
       </c>
@@ -26426,7 +26459,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="454" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="454" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A454" s="1" t="b">
         <v>0</v>
       </c>
@@ -26470,7 +26503,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="455" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="455" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A455" s="1" t="b">
         <v>0</v>
       </c>
@@ -26514,7 +26547,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="456" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="456" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A456" s="1" t="b">
         <v>0</v>
       </c>
@@ -26558,9 +26591,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="457" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A457" s="1" t="b">
-        <v>0</v>
+    <row r="457" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A457" s="6" t="s">
+        <v>2008</v>
       </c>
       <c r="B457" s="3">
         <v>273010</v>
@@ -26602,7 +26635,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="458" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="458" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A458" s="1" t="b">
         <v>0</v>
       </c>
@@ -26646,9 +26679,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="459" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A459" s="1" t="b">
-        <v>0</v>
+    <row r="459" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A459" s="6" t="s">
+        <v>2010</v>
       </c>
       <c r="B459" s="3">
         <v>273030</v>
@@ -26690,7 +26723,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="460" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="460" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A460" s="1" t="b">
         <v>0</v>
       </c>
@@ -26734,7 +26767,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="461" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="461" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A461" s="1" t="b">
         <v>0</v>
       </c>
@@ -26778,7 +26811,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="462" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="462" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A462" s="1" t="b">
         <v>0</v>
       </c>
@@ -26822,7 +26855,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="463" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="463" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A463" s="1" t="b">
         <v>0</v>
       </c>
@@ -66014,6 +66047,17 @@
     <hyperlink ref="A905" r:id="rId1343" xr:uid="{6F69D3AA-AEA7-1142-9894-0755A8D901C0}"/>
     <hyperlink ref="B905" r:id="rId1344" display="https://volcano.si.edu/volcano.cfm?vn=332010" xr:uid="{49AFC9C8-A551-3948-9FE3-436253A7BFE1}"/>
     <hyperlink ref="A904" r:id="rId1345" display="https://insarmaps.miami.edu/start/19.4032/-155.2273/10.9779?flyToDatasetCenter=false&amp;startDataset=S1_vert_087_124_mintpy_20180902_XXXXXXXX_N1978W15586_N1978W15473_N1912W15473_N1912W15586&amp;pointLat=19.39940&amp;pointLon=-155.27805&amp;minScale=-20&amp;maxScale=20&amp;startDate=20180902&amp;endDate=20260228&amp;pixelSize=3.3" xr:uid="{06950C1A-A714-B24B-BABA-AC6C3B02267A}"/>
+    <hyperlink ref="A401" r:id="rId1346" display="http://149.165.154.65/data/HDF5EOS/Lewotolok/miaiply" xr:uid="{73831688-CC6A-3643-8C99-1F23A35EC407}"/>
+    <hyperlink ref="A398" r:id="rId1347" location="/start/-8.5402/122.7753/13.5@minScale=-1.5&amp;maxScale=1.5" xr:uid="{BA612BF8-6BAA-CB4E-9663-BCA3638E8A15}"/>
+    <hyperlink ref="A349" r:id="rId1348" location="/start/-1.696/101.270/14.4?minScale=-0.8&amp;maxScale=0.8&amp;background=satellite" xr:uid="{38CAB67B-7C95-0943-9B63-ECFFB44BCC04}"/>
+    <hyperlink ref="A396" r:id="rId1349" display="http://149.165.153.50/start/-8.2450/117.9958/12.5292?flyToDatasetCenter=false&amp;startDataset=S1_asc_083_miaplpy_20141023_20250215_S0836E11794_S0832E11809_S0817E11806_S0820E11792_filtDel4DS&amp;minScale=-3&amp;maxScale=3&amp;startDate=20141023&amp;endDate=20250215&amp;pixelSize=2.1&amp;background=satellite" xr:uid="{074096C7-BC89-3546-B9E6-FF4457770D48}"/>
+    <hyperlink ref="A395" r:id="rId1350" location="/?minScale=-2&amp;maxScale=2" xr:uid="{F3B432C2-873D-E449-9307-C22F5E984A00}"/>
+    <hyperlink ref="A394" r:id="rId1351" location="/?minScale=-2&amp;maxScale=2" xr:uid="{9CDE4C14-CEA9-B04D-B9EC-D9486F8733A6}"/>
+    <hyperlink ref="A457" r:id="rId1352" location="/?minScale=-2&amp;maxScale=2&amp;background=satellite" xr:uid="{A0F91AE9-8E31-0D4A-96E8-81CCF82F1A52}"/>
+    <hyperlink ref="A383" r:id="rId1353" location="/?minScale=-3&amp;maxScale=3&amp;background=satellite" xr:uid="{D1B95BF0-B5D7-D447-B1AA-4DF1E4361020}"/>
+    <hyperlink ref="A459" r:id="rId1354" location="/?minScale=-2&amp;maxScale=2" xr:uid="{979264A1-1EDE-9941-B821-5E19B7EC19AE}"/>
+    <hyperlink ref="A338" r:id="rId1355" location="/?minScale=-5&amp;maxScale=5&amp;background=satellite" xr:uid="{B59A7083-C90A-3442-B482-B97C567E58E3}"/>
+    <hyperlink ref="A385" r:id="rId1356" location="/?minScale=-2&amp;maxScale=2" xr:uid="{ADDB8508-D649-ED42-98CC-A33FD8E3B0DE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>